<commit_message>
added mounting holes and produced manufacturing files, ALL IS DONE Alhamdulillah
</commit_message>
<xml_diff>
--- a/Documents/jlc_PNP.xlsx
+++ b/Documents/jlc_PNP.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="159">
   <si>
     <t xml:space="preserve">Designator</t>
   </si>
@@ -37,15 +37,12 @@
     <t xml:space="preserve">Rotation</t>
   </si>
   <si>
-    <t xml:space="preserve">Amb</t>
+    <t xml:space="preserve">C203</t>
   </si>
   <si>
     <t xml:space="preserve">bottom</t>
   </si>
   <si>
-    <t xml:space="preserve">C203</t>
-  </si>
-  <si>
     <t xml:space="preserve">C204</t>
   </si>
   <si>
@@ -118,9 +115,6 @@
     <t xml:space="preserve">PS501</t>
   </si>
   <si>
-    <t xml:space="preserve">Pipe</t>
-  </si>
-  <si>
     <t xml:space="preserve">R203</t>
   </si>
   <si>
@@ -166,6 +160,12 @@
     <t xml:space="preserve">R611</t>
   </si>
   <si>
+    <t xml:space="preserve">TP601</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TP602</t>
+  </si>
+  <si>
     <t xml:space="preserve">U401</t>
   </si>
   <si>
@@ -178,21 +178,12 @@
     <t xml:space="preserve">U602</t>
   </si>
   <si>
-    <t xml:space="preserve">3V3</t>
+    <t xml:space="preserve">C201</t>
   </si>
   <si>
     <t xml:space="preserve">top</t>
   </si>
   <si>
-    <t xml:space="preserve">3V3 F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C201</t>
-  </si>
-  <si>
     <t xml:space="preserve">C202</t>
   </si>
   <si>
@@ -205,6 +196,75 @@
     <t xml:space="preserve">C213</t>
   </si>
   <si>
+    <t xml:space="preserve">C301</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C302</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C303</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C304</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C305</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C306</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C307</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C308</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C309</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C310</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C311</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C312</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C313</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C314</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C315</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C316</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C317</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C318</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C319</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C320</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C321</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C322</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C323</t>
+  </si>
+  <si>
     <t xml:space="preserve">C504</t>
   </si>
   <si>
@@ -247,31 +307,31 @@
     <t xml:space="preserve">FB501</t>
   </si>
   <si>
-    <t xml:space="preserve">FL301</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FL302</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FL303</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HUMIDITY</t>
-  </si>
-  <si>
     <t xml:space="preserve">J201</t>
   </si>
   <si>
     <t xml:space="preserve">J202</t>
   </si>
   <si>
+    <t xml:space="preserve">J203</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J205</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J206</t>
+  </si>
+  <si>
     <t xml:space="preserve">J301</t>
   </si>
   <si>
-    <t xml:space="preserve">J302</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J303</t>
+    <t xml:space="preserve">J304</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J305</t>
   </si>
   <si>
     <t xml:space="preserve">J501</t>
@@ -295,7 +355,73 @@
     <t xml:space="preserve">J602</t>
   </si>
   <si>
-    <t xml:space="preserve">PRESSURE</t>
+    <t xml:space="preserve">J603</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J604</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L301</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L302</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L303</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L304</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L305</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L306</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L307</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L308</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L309</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L310</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L311</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L312</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L313</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L314</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L315</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L316</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L317</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L318</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L319</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L320</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L321</t>
   </si>
   <si>
     <t xml:space="preserve">R201</t>
@@ -352,22 +478,19 @@
     <t xml:space="preserve">R509</t>
   </si>
   <si>
+    <t xml:space="preserve">TP501</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TP502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TP503</t>
+  </si>
+  <si>
     <t xml:space="preserve">U201</t>
   </si>
   <si>
     <t xml:space="preserve">U202</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UART1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UART2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UART3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UART4</t>
   </si>
   <si>
     <t xml:space="preserve">Y201</t>
@@ -388,6 +511,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -469,14 +593,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E112"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E153"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="7.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="5.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="5.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="7.13"/>
   </cols>
   <sheetData>
@@ -502,16 +626,16 @@
         <v>5</v>
       </c>
       <c r="B2" s="0" t="n">
-        <v>149.225</v>
+        <v>152.320893</v>
       </c>
       <c r="C2" s="0" t="n">
-        <v>-105.025</v>
+        <v>-114.468915</v>
       </c>
       <c r="D2" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E2" s="0" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -519,16 +643,16 @@
         <v>7</v>
       </c>
       <c r="B3" s="0" t="n">
-        <v>152.320893</v>
+        <v>149.370389</v>
       </c>
       <c r="C3" s="0" t="n">
-        <v>-114.468915</v>
+        <v>-121.539</v>
       </c>
       <c r="D3" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E3" s="0" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -536,16 +660,16 @@
         <v>8</v>
       </c>
       <c r="B4" s="0" t="n">
-        <v>149.370389</v>
+        <v>149.479</v>
       </c>
       <c r="C4" s="0" t="n">
-        <v>-121.539</v>
+        <v>-119.634</v>
       </c>
       <c r="D4" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E4" s="0" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -553,16 +677,16 @@
         <v>9</v>
       </c>
       <c r="B5" s="0" t="n">
-        <v>149.479</v>
+        <v>145.034</v>
       </c>
       <c r="C5" s="0" t="n">
-        <v>-119.634</v>
+        <v>-122.174</v>
       </c>
       <c r="D5" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E5" s="0" t="n">
-        <v>180</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -570,16 +694,16 @@
         <v>10</v>
       </c>
       <c r="B6" s="0" t="n">
-        <v>145.034</v>
+        <v>146.431</v>
       </c>
       <c r="C6" s="0" t="n">
-        <v>-122.174</v>
+        <v>-117.729</v>
       </c>
       <c r="D6" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E6" s="0" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -587,10 +711,10 @@
         <v>11</v>
       </c>
       <c r="B7" s="0" t="n">
-        <v>146.431</v>
+        <v>148.209</v>
       </c>
       <c r="C7" s="0" t="n">
-        <v>-117.729</v>
+        <v>-111.76</v>
       </c>
       <c r="D7" s="0" t="s">
         <v>6</v>
@@ -604,16 +728,16 @@
         <v>12</v>
       </c>
       <c r="B8" s="0" t="n">
-        <v>148.209</v>
+        <v>152.654</v>
       </c>
       <c r="C8" s="0" t="n">
-        <v>-111.76</v>
+        <v>-120.65</v>
       </c>
       <c r="D8" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E8" s="0" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -621,10 +745,10 @@
         <v>13</v>
       </c>
       <c r="B9" s="0" t="n">
-        <v>152.654</v>
+        <v>152.4</v>
       </c>
       <c r="C9" s="0" t="n">
-        <v>-120.65</v>
+        <v>-115.951</v>
       </c>
       <c r="D9" s="0" t="s">
         <v>6</v>
@@ -638,16 +762,16 @@
         <v>14</v>
       </c>
       <c r="B10" s="0" t="n">
-        <v>152.4</v>
+        <v>159.8</v>
       </c>
       <c r="C10" s="0" t="n">
-        <v>-115.951</v>
+        <v>-119</v>
       </c>
       <c r="D10" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E10" s="0" t="n">
-        <v>180</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -655,10 +779,10 @@
         <v>15</v>
       </c>
       <c r="B11" s="0" t="n">
-        <v>159.8</v>
+        <v>167.6</v>
       </c>
       <c r="C11" s="0" t="n">
-        <v>-119</v>
+        <v>-129.025</v>
       </c>
       <c r="D11" s="0" t="s">
         <v>6</v>
@@ -672,10 +796,10 @@
         <v>16</v>
       </c>
       <c r="B12" s="0" t="n">
-        <v>167.6</v>
+        <v>165.8</v>
       </c>
       <c r="C12" s="0" t="n">
-        <v>-129.025</v>
+        <v>-129.225</v>
       </c>
       <c r="D12" s="0" t="s">
         <v>6</v>
@@ -689,7 +813,7 @@
         <v>17</v>
       </c>
       <c r="B13" s="0" t="n">
-        <v>165.8</v>
+        <v>163.8</v>
       </c>
       <c r="C13" s="0" t="n">
         <v>-129.225</v>
@@ -706,16 +830,16 @@
         <v>18</v>
       </c>
       <c r="B14" s="0" t="n">
-        <v>163.8</v>
+        <v>165.3</v>
       </c>
       <c r="C14" s="0" t="n">
-        <v>-129.225</v>
+        <v>-118.11</v>
       </c>
       <c r="D14" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E14" s="0" t="n">
-        <v>-90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -723,16 +847,16 @@
         <v>19</v>
       </c>
       <c r="B15" s="0" t="n">
-        <v>165.3</v>
+        <v>168.8</v>
       </c>
       <c r="C15" s="0" t="n">
-        <v>-118.11</v>
+        <v>-120</v>
       </c>
       <c r="D15" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E15" s="0" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -743,7 +867,7 @@
         <v>168.8</v>
       </c>
       <c r="C16" s="0" t="n">
-        <v>-120</v>
+        <v>-122</v>
       </c>
       <c r="D16" s="0" t="s">
         <v>6</v>
@@ -757,16 +881,16 @@
         <v>21</v>
       </c>
       <c r="B17" s="0" t="n">
-        <v>168.8</v>
+        <v>165.575</v>
       </c>
       <c r="C17" s="0" t="n">
-        <v>-122</v>
+        <v>-120.396</v>
       </c>
       <c r="D17" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E17" s="0" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -774,16 +898,16 @@
         <v>22</v>
       </c>
       <c r="B18" s="0" t="n">
-        <v>165.575</v>
+        <v>162.3</v>
       </c>
       <c r="C18" s="0" t="n">
-        <v>-120.396</v>
+        <v>-114</v>
       </c>
       <c r="D18" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E18" s="0" t="n">
-        <v>180</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -791,16 +915,16 @@
         <v>23</v>
       </c>
       <c r="B19" s="0" t="n">
-        <v>162.3</v>
+        <v>158.496</v>
       </c>
       <c r="C19" s="0" t="n">
-        <v>-114</v>
+        <v>-113.665</v>
       </c>
       <c r="D19" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E19" s="0" t="n">
-        <v>90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -808,16 +932,16 @@
         <v>24</v>
       </c>
       <c r="B20" s="0" t="n">
-        <v>158.496</v>
+        <v>162.3</v>
       </c>
       <c r="C20" s="0" t="n">
-        <v>-113.665</v>
+        <v>-110.6</v>
       </c>
       <c r="D20" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E20" s="0" t="n">
-        <v>180</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -825,16 +949,16 @@
         <v>25</v>
       </c>
       <c r="B21" s="0" t="n">
-        <v>162.3</v>
+        <v>151.638</v>
       </c>
       <c r="C21" s="0" t="n">
-        <v>-110.6</v>
+        <v>-106.045</v>
       </c>
       <c r="D21" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E21" s="0" t="n">
-        <v>-90</v>
+        <v>90</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -842,16 +966,16 @@
         <v>26</v>
       </c>
       <c r="B22" s="0" t="n">
-        <v>151.638</v>
+        <v>145.625</v>
       </c>
       <c r="C22" s="0" t="n">
-        <v>-106.045</v>
+        <v>-105.225</v>
       </c>
       <c r="D22" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E22" s="0" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -859,16 +983,16 @@
         <v>27</v>
       </c>
       <c r="B23" s="0" t="n">
-        <v>145.625</v>
+        <v>129.01</v>
       </c>
       <c r="C23" s="0" t="n">
-        <v>-105.225</v>
+        <v>-124.206</v>
       </c>
       <c r="D23" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E23" s="0" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -876,16 +1000,16 @@
         <v>28</v>
       </c>
       <c r="B24" s="0" t="n">
-        <v>129.01</v>
+        <v>128.982</v>
       </c>
       <c r="C24" s="0" t="n">
-        <v>-124.206</v>
+        <v>-104.521</v>
       </c>
       <c r="D24" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E24" s="0" t="n">
-        <v>90</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -893,16 +1017,16 @@
         <v>29</v>
       </c>
       <c r="B25" s="0" t="n">
-        <v>128.982</v>
+        <v>148.844</v>
       </c>
       <c r="C25" s="0" t="n">
-        <v>-104.521</v>
+        <v>-117.1375</v>
       </c>
       <c r="D25" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E25" s="0" t="n">
-        <v>-90</v>
+        <v>90</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -910,16 +1034,16 @@
         <v>30</v>
       </c>
       <c r="B26" s="0" t="n">
-        <v>148.844</v>
+        <v>165.35</v>
       </c>
       <c r="C26" s="0" t="n">
-        <v>-117.1375</v>
+        <v>-125.225</v>
       </c>
       <c r="D26" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E26" s="0" t="n">
-        <v>90</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -927,16 +1051,16 @@
         <v>31</v>
       </c>
       <c r="B27" s="0" t="n">
-        <v>165.35</v>
+        <v>153.67</v>
       </c>
       <c r="C27" s="0" t="n">
-        <v>-125.225</v>
+        <v>-117.602</v>
       </c>
       <c r="D27" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E27" s="0" t="n">
-        <v>-90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -944,10 +1068,10 @@
         <v>32</v>
       </c>
       <c r="B28" s="0" t="n">
-        <v>141.4</v>
+        <v>153.797</v>
       </c>
       <c r="C28" s="0" t="n">
-        <v>-106.225</v>
+        <v>-119.126</v>
       </c>
       <c r="D28" s="0" t="s">
         <v>6</v>
@@ -961,16 +1085,16 @@
         <v>33</v>
       </c>
       <c r="B29" s="0" t="n">
-        <v>153.67</v>
+        <v>161.8</v>
       </c>
       <c r="C29" s="0" t="n">
-        <v>-117.602</v>
+        <v>-123.85</v>
       </c>
       <c r="D29" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E29" s="0" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -978,16 +1102,16 @@
         <v>34</v>
       </c>
       <c r="B30" s="0" t="n">
-        <v>153.797</v>
+        <v>159.512</v>
       </c>
       <c r="C30" s="0" t="n">
-        <v>-119.126</v>
+        <v>-123.063</v>
       </c>
       <c r="D30" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E30" s="0" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -998,13 +1122,13 @@
         <v>161.8</v>
       </c>
       <c r="C31" s="0" t="n">
-        <v>-123.85</v>
+        <v>-127.225</v>
       </c>
       <c r="D31" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E31" s="0" t="n">
-        <v>90</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1012,10 +1136,10 @@
         <v>36</v>
       </c>
       <c r="B32" s="0" t="n">
-        <v>159.512</v>
+        <v>165.354</v>
       </c>
       <c r="C32" s="0" t="n">
-        <v>-123.063</v>
+        <v>-121.92</v>
       </c>
       <c r="D32" s="0" t="s">
         <v>6</v>
@@ -1029,16 +1153,16 @@
         <v>37</v>
       </c>
       <c r="B33" s="0" t="n">
-        <v>161.8</v>
+        <v>163.068</v>
       </c>
       <c r="C33" s="0" t="n">
-        <v>-127.225</v>
+        <v>-120.65</v>
       </c>
       <c r="D33" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E33" s="0" t="n">
-        <v>-90</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1046,16 +1170,16 @@
         <v>38</v>
       </c>
       <c r="B34" s="0" t="n">
-        <v>165.354</v>
+        <v>139.2</v>
       </c>
       <c r="C34" s="0" t="n">
-        <v>-121.92</v>
+        <v>-100.2375</v>
       </c>
       <c r="D34" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E34" s="0" t="n">
-        <v>180</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1063,16 +1187,16 @@
         <v>39</v>
       </c>
       <c r="B35" s="0" t="n">
-        <v>163.068</v>
+        <v>136.825</v>
       </c>
       <c r="C35" s="0" t="n">
-        <v>-120.65</v>
+        <v>-104.025</v>
       </c>
       <c r="D35" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E35" s="0" t="n">
-        <v>90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1080,16 +1204,16 @@
         <v>40</v>
       </c>
       <c r="B36" s="0" t="n">
-        <v>139.2</v>
+        <v>136.8</v>
       </c>
       <c r="C36" s="0" t="n">
-        <v>-100.2375</v>
+        <v>-102.425</v>
       </c>
       <c r="D36" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E36" s="0" t="n">
-        <v>-90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1097,16 +1221,16 @@
         <v>41</v>
       </c>
       <c r="B37" s="0" t="n">
-        <v>136.825</v>
+        <v>139.2</v>
       </c>
       <c r="C37" s="0" t="n">
-        <v>-104.025</v>
+        <v>-103.2375</v>
       </c>
       <c r="D37" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E37" s="0" t="n">
-        <v>180</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1114,16 +1238,16 @@
         <v>42</v>
       </c>
       <c r="B38" s="0" t="n">
-        <v>136.8</v>
+        <v>148.6</v>
       </c>
       <c r="C38" s="0" t="n">
-        <v>-102.425</v>
+        <v>-102.025</v>
       </c>
       <c r="D38" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E38" s="0" t="n">
-        <v>0</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1131,16 +1255,16 @@
         <v>43</v>
       </c>
       <c r="B39" s="0" t="n">
-        <v>139.2</v>
+        <v>151</v>
       </c>
       <c r="C39" s="0" t="n">
-        <v>-103.2375</v>
+        <v>-101.225</v>
       </c>
       <c r="D39" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E39" s="0" t="n">
-        <v>-90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1148,16 +1272,16 @@
         <v>44</v>
       </c>
       <c r="B40" s="0" t="n">
-        <v>148.6</v>
+        <v>151</v>
       </c>
       <c r="C40" s="0" t="n">
-        <v>-102.025</v>
+        <v>-102.825</v>
       </c>
       <c r="D40" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E40" s="0" t="n">
-        <v>-90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1165,16 +1289,16 @@
         <v>45</v>
       </c>
       <c r="B41" s="0" t="n">
-        <v>151</v>
+        <v>148.6</v>
       </c>
       <c r="C41" s="0" t="n">
-        <v>-101.225</v>
+        <v>-99.025</v>
       </c>
       <c r="D41" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E41" s="0" t="n">
-        <v>0</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1182,16 +1306,16 @@
         <v>46</v>
       </c>
       <c r="B42" s="0" t="n">
-        <v>151</v>
+        <v>141.4</v>
       </c>
       <c r="C42" s="0" t="n">
-        <v>-102.825</v>
+        <v>-106.225</v>
       </c>
       <c r="D42" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E42" s="0" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1199,16 +1323,16 @@
         <v>47</v>
       </c>
       <c r="B43" s="0" t="n">
-        <v>148.6</v>
+        <v>149.225</v>
       </c>
       <c r="C43" s="0" t="n">
-        <v>-99.025</v>
+        <v>-105.025</v>
       </c>
       <c r="D43" s="0" t="s">
         <v>6</v>
       </c>
       <c r="E43" s="0" t="n">
-        <v>-90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1284,16 +1408,16 @@
         <v>52</v>
       </c>
       <c r="B48" s="0" t="n">
-        <v>167</v>
+        <v>143.166726</v>
       </c>
       <c r="C48" s="0" t="n">
-        <v>-107.1</v>
+        <v>-122</v>
       </c>
       <c r="D48" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E48" s="0" t="n">
-        <v>180</v>
+        <v>-135</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1301,16 +1425,16 @@
         <v>54</v>
       </c>
       <c r="B49" s="0" t="n">
-        <v>156.3</v>
+        <v>155.455478</v>
       </c>
       <c r="C49" s="0" t="n">
-        <v>-103.1</v>
+        <v>-126.565157</v>
       </c>
       <c r="D49" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E49" s="0" t="n">
-        <v>180</v>
+        <v>-55</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1318,16 +1442,16 @@
         <v>55</v>
       </c>
       <c r="B50" s="0" t="n">
-        <v>168.9</v>
+        <v>154.155478</v>
       </c>
       <c r="C50" s="0" t="n">
-        <v>-117.7</v>
+        <v>-127.465157</v>
       </c>
       <c r="D50" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E50" s="0" t="n">
-        <v>180</v>
+        <v>-55</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1335,16 +1459,16 @@
         <v>56</v>
       </c>
       <c r="B51" s="0" t="n">
-        <v>143.166726</v>
+        <v>143.256</v>
       </c>
       <c r="C51" s="0" t="n">
-        <v>-122</v>
+        <v>-118.491</v>
       </c>
       <c r="D51" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E51" s="0" t="n">
-        <v>-135</v>
+        <v>135</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1352,16 +1476,16 @@
         <v>57</v>
       </c>
       <c r="B52" s="0" t="n">
-        <v>154.2</v>
+        <v>162.575</v>
       </c>
       <c r="C52" s="0" t="n">
-        <v>-122.6</v>
+        <v>-105.975</v>
       </c>
       <c r="D52" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E52" s="0" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1369,16 +1493,16 @@
         <v>58</v>
       </c>
       <c r="B53" s="0" t="n">
-        <v>151.6</v>
+        <v>141.535702</v>
       </c>
       <c r="C53" s="0" t="n">
-        <v>-124.4</v>
+        <v>-128.12039</v>
       </c>
       <c r="D53" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E53" s="0" t="n">
-        <v>-145</v>
+        <v>-125</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1386,16 +1510,16 @@
         <v>59</v>
       </c>
       <c r="B54" s="0" t="n">
-        <v>143.256</v>
+        <v>138.824583</v>
       </c>
       <c r="C54" s="0" t="n">
-        <v>-118.491</v>
+        <v>-130.20553</v>
       </c>
       <c r="D54" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E54" s="0" t="n">
-        <v>135</v>
+        <v>-35</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1403,16 +1527,16 @@
         <v>60</v>
       </c>
       <c r="B55" s="0" t="n">
-        <v>162.575</v>
+        <v>137.218569</v>
       </c>
       <c r="C55" s="0" t="n">
-        <v>-105.975</v>
+        <v>-132.499155</v>
       </c>
       <c r="D55" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E55" s="0" t="n">
-        <v>0</v>
+        <v>-35</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1420,16 +1544,16 @@
         <v>61</v>
       </c>
       <c r="B56" s="0" t="n">
-        <v>169.735</v>
+        <v>147.074294</v>
       </c>
       <c r="C56" s="0" t="n">
-        <v>-131.265</v>
+        <v>-129.966867</v>
       </c>
       <c r="D56" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E56" s="0" t="n">
-        <v>0</v>
+        <v>-105</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1437,16 +1561,16 @@
         <v>62</v>
       </c>
       <c r="B57" s="0" t="n">
-        <v>156.3</v>
+        <v>141.126367</v>
       </c>
       <c r="C57" s="0" t="n">
-        <v>-101.2</v>
+        <v>-126.124684</v>
       </c>
       <c r="D57" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E57" s="0" t="n">
-        <v>180</v>
+        <v>-35</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1454,16 +1578,16 @@
         <v>63</v>
       </c>
       <c r="B58" s="0" t="n">
-        <v>130.7</v>
+        <v>136.825139</v>
       </c>
       <c r="C58" s="0" t="n">
-        <v>-101.3</v>
+        <v>-133.932757</v>
       </c>
       <c r="D58" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E58" s="0" t="n">
-        <v>0</v>
+        <v>-125</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1471,16 +1595,16 @@
         <v>64</v>
       </c>
       <c r="B59" s="0" t="n">
-        <v>158.6</v>
+        <v>142.302463</v>
       </c>
       <c r="C59" s="0" t="n">
-        <v>-128</v>
+        <v>-128.713583</v>
       </c>
       <c r="D59" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E59" s="0" t="n">
-        <v>0</v>
+        <v>-125</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1488,16 +1612,16 @@
         <v>65</v>
       </c>
       <c r="B60" s="0" t="n">
-        <v>169.6</v>
+        <v>145.136356</v>
       </c>
       <c r="C60" s="0" t="n">
-        <v>-129</v>
+        <v>-127.875767</v>
       </c>
       <c r="D60" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E60" s="0" t="n">
-        <v>180</v>
+        <v>-15</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1505,16 +1629,16 @@
         <v>66</v>
       </c>
       <c r="B61" s="0" t="n">
-        <v>169.8</v>
+        <v>146.121309</v>
       </c>
       <c r="C61" s="0" t="n">
-        <v>-123.825</v>
+        <v>-129.659752</v>
       </c>
       <c r="D61" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E61" s="0" t="n">
-        <v>90</v>
+        <v>-105</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1522,16 +1646,16 @@
         <v>67</v>
       </c>
       <c r="B62" s="0" t="n">
-        <v>153.7</v>
+        <v>144.920616</v>
       </c>
       <c r="C62" s="0" t="n">
-        <v>-105.925</v>
+        <v>-133.781705</v>
       </c>
       <c r="D62" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E62" s="0" t="n">
-        <v>90</v>
+        <v>165</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1539,16 +1663,16 @@
         <v>68</v>
       </c>
       <c r="B63" s="0" t="n">
-        <v>167.25</v>
+        <v>144.1</v>
       </c>
       <c r="C63" s="0" t="n">
-        <v>-113.325</v>
+        <v>-136.5</v>
       </c>
       <c r="D63" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E63" s="0" t="n">
-        <v>90</v>
+        <v>165</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1556,16 +1680,16 @@
         <v>69</v>
       </c>
       <c r="B64" s="0" t="n">
-        <v>124.206</v>
+        <v>143.3</v>
       </c>
       <c r="C64" s="0" t="n">
-        <v>-96.393</v>
+        <v>-137.7</v>
       </c>
       <c r="D64" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E64" s="0" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1573,16 +1697,16 @@
         <v>70</v>
       </c>
       <c r="B65" s="0" t="n">
-        <v>124</v>
+        <v>144.75</v>
       </c>
       <c r="C65" s="0" t="n">
-        <v>-141.4</v>
+        <v>-130.75</v>
       </c>
       <c r="D65" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E65" s="0" t="n">
-        <v>0</v>
+        <v>-15</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1590,16 +1714,16 @@
         <v>71</v>
       </c>
       <c r="B66" s="0" t="n">
-        <v>174.6</v>
+        <v>146.598616</v>
       </c>
       <c r="C66" s="0" t="n">
-        <v>-96.75</v>
+        <v>-126.16381</v>
       </c>
       <c r="D66" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E66" s="0" t="n">
-        <v>180</v>
+        <v>165</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1607,16 +1731,16 @@
         <v>72</v>
       </c>
       <c r="B67" s="0" t="n">
-        <v>174.4</v>
+        <v>149.274081</v>
       </c>
       <c r="C67" s="0" t="n">
-        <v>-141.4</v>
+        <v>-130.067736</v>
       </c>
       <c r="D67" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E67" s="0" t="n">
-        <v>180</v>
+        <v>15</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1624,16 +1748,16 @@
         <v>73</v>
       </c>
       <c r="B68" s="0" t="n">
-        <v>165.6</v>
+        <v>149.034581</v>
       </c>
       <c r="C68" s="0" t="n">
-        <v>-135.4</v>
+        <v>-129.096634</v>
       </c>
       <c r="D68" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E68" s="0" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1641,16 +1765,16 @@
         <v>74</v>
       </c>
       <c r="B69" s="0" t="n">
-        <v>158.7</v>
+        <v>151.557628</v>
       </c>
       <c r="C69" s="0" t="n">
-        <v>-115.5</v>
+        <v>-127.385309</v>
       </c>
       <c r="D69" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E69" s="0" t="n">
-        <v>180</v>
+        <v>-165</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1658,16 +1782,16 @@
         <v>75</v>
       </c>
       <c r="B70" s="0" t="n">
-        <v>138.651332</v>
+        <v>150.471086</v>
       </c>
       <c r="C70" s="0" t="n">
-        <v>-132.190412</v>
+        <v>-129.125834</v>
       </c>
       <c r="D70" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E70" s="0" t="n">
-        <v>180</v>
+        <v>-75</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1675,16 +1799,16 @@
         <v>76</v>
       </c>
       <c r="B71" s="0" t="n">
-        <v>144.384</v>
+        <v>151.194485</v>
       </c>
       <c r="C71" s="0" t="n">
-        <v>-133</v>
+        <v>-131.825597</v>
       </c>
       <c r="D71" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E71" s="0" t="n">
-        <v>180</v>
+        <v>-75</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1692,16 +1816,16 @@
         <v>77</v>
       </c>
       <c r="B72" s="0" t="n">
-        <v>151.103984</v>
+        <v>152.35</v>
       </c>
       <c r="C72" s="0" t="n">
-        <v>-132.5</v>
+        <v>-135.887315</v>
       </c>
       <c r="D72" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E72" s="0" t="n">
-        <v>-135</v>
+        <v>15</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1709,16 +1833,16 @@
         <v>78</v>
       </c>
       <c r="B73" s="0" t="n">
-        <v>131.182</v>
+        <v>151.65</v>
       </c>
       <c r="C73" s="0" t="n">
-        <v>-112.732</v>
+        <v>-133.182722</v>
       </c>
       <c r="D73" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E73" s="0" t="n">
-        <v>90</v>
+        <v>15</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1726,16 +1850,16 @@
         <v>79</v>
       </c>
       <c r="B74" s="0" t="n">
-        <v>150.876</v>
+        <v>153.133305</v>
       </c>
       <c r="C74" s="0" t="n">
-        <v>-93.472</v>
+        <v>-137.12952</v>
       </c>
       <c r="D74" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E74" s="0" t="n">
-        <v>-90</v>
+        <v>105</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1743,16 +1867,16 @@
         <v>80</v>
       </c>
       <c r="B75" s="0" t="n">
-        <v>163.595</v>
+        <v>151.799359</v>
       </c>
       <c r="C75" s="0" t="n">
-        <v>-98.825</v>
+        <v>-130.219311</v>
       </c>
       <c r="D75" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E75" s="0" t="n">
-        <v>180</v>
+        <v>-165</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1760,16 +1884,16 @@
         <v>81</v>
       </c>
       <c r="B76" s="0" t="n">
-        <v>134.86</v>
+        <v>169.735</v>
       </c>
       <c r="C76" s="0" t="n">
-        <v>-139.94</v>
+        <v>-131.265</v>
       </c>
       <c r="D76" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E76" s="0" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1777,10 +1901,10 @@
         <v>82</v>
       </c>
       <c r="B77" s="0" t="n">
-        <v>143.6</v>
+        <v>156.3</v>
       </c>
       <c r="C77" s="0" t="n">
-        <v>-140</v>
+        <v>-101.2</v>
       </c>
       <c r="D77" s="0" t="s">
         <v>53</v>
@@ -1794,16 +1918,16 @@
         <v>83</v>
       </c>
       <c r="B78" s="0" t="n">
-        <v>152.5</v>
+        <v>130.7</v>
       </c>
       <c r="C78" s="0" t="n">
-        <v>-140</v>
+        <v>-101.3</v>
       </c>
       <c r="D78" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E78" s="0" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1811,16 +1935,16 @@
         <v>84</v>
       </c>
       <c r="B79" s="0" t="n">
-        <v>122.3877</v>
+        <v>158.6</v>
       </c>
       <c r="C79" s="0" t="n">
-        <v>-103.35</v>
+        <v>-128</v>
       </c>
       <c r="D79" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E79" s="0" t="n">
-        <v>-90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1828,16 +1952,16 @@
         <v>85</v>
       </c>
       <c r="B80" s="0" t="n">
-        <v>122.3</v>
+        <v>169.6</v>
       </c>
       <c r="C80" s="0" t="n">
-        <v>-129.9</v>
+        <v>-129</v>
       </c>
       <c r="D80" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E80" s="0" t="n">
-        <v>-90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1845,10 +1969,10 @@
         <v>86</v>
       </c>
       <c r="B81" s="0" t="n">
-        <v>176.1675</v>
+        <v>169.8</v>
       </c>
       <c r="C81" s="0" t="n">
-        <v>-108.25</v>
+        <v>-123.825</v>
       </c>
       <c r="D81" s="0" t="s">
         <v>53</v>
@@ -1862,10 +1986,10 @@
         <v>87</v>
       </c>
       <c r="B82" s="0" t="n">
-        <v>176.1754</v>
+        <v>153.7</v>
       </c>
       <c r="C82" s="0" t="n">
-        <v>-134.6</v>
+        <v>-105.925</v>
       </c>
       <c r="D82" s="0" t="s">
         <v>53</v>
@@ -1879,16 +2003,16 @@
         <v>88</v>
       </c>
       <c r="B83" s="0" t="n">
-        <v>160.85</v>
+        <v>167.25</v>
       </c>
       <c r="C83" s="0" t="n">
-        <v>-142.8675</v>
+        <v>-113.325</v>
       </c>
       <c r="D83" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E83" s="0" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1896,16 +2020,16 @@
         <v>89</v>
       </c>
       <c r="B84" s="0" t="n">
-        <v>134.116</v>
+        <v>124.206</v>
       </c>
       <c r="C84" s="0" t="n">
-        <v>-98.716</v>
+        <v>-96.393</v>
       </c>
       <c r="D84" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E84" s="0" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1913,16 +2037,16 @@
         <v>90</v>
       </c>
       <c r="B85" s="0" t="n">
-        <v>157.103</v>
+        <v>124</v>
       </c>
       <c r="C85" s="0" t="n">
-        <v>-98.843</v>
+        <v>-141.4</v>
       </c>
       <c r="D85" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E85" s="0" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1930,16 +2054,16 @@
         <v>91</v>
       </c>
       <c r="B86" s="0" t="n">
-        <v>131.2</v>
+        <v>174.6</v>
       </c>
       <c r="C86" s="0" t="n">
-        <v>-130.389</v>
+        <v>-96.75</v>
       </c>
       <c r="D86" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E86" s="0" t="n">
-        <v>90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1947,16 +2071,16 @@
         <v>92</v>
       </c>
       <c r="B87" s="0" t="n">
-        <v>139.7</v>
+        <v>174.4</v>
       </c>
       <c r="C87" s="0" t="n">
-        <v>-112.649</v>
+        <v>-141.4</v>
       </c>
       <c r="D87" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E87" s="0" t="n">
-        <v>-45</v>
+        <v>180</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1964,16 +2088,16 @@
         <v>93</v>
       </c>
       <c r="B88" s="0" t="n">
-        <v>138.557</v>
+        <v>165.6</v>
       </c>
       <c r="C88" s="0" t="n">
-        <v>-113.792</v>
+        <v>-135.4</v>
       </c>
       <c r="D88" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E88" s="0" t="n">
-        <v>-45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1981,16 +2105,16 @@
         <v>94</v>
       </c>
       <c r="B89" s="0" t="n">
-        <v>158.6</v>
+        <v>158.7</v>
       </c>
       <c r="C89" s="0" t="n">
-        <v>-126.2</v>
+        <v>-115.5</v>
       </c>
       <c r="D89" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E89" s="0" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1998,10 +2122,10 @@
         <v>95</v>
       </c>
       <c r="B90" s="0" t="n">
-        <v>150.622</v>
+        <v>150.876</v>
       </c>
       <c r="C90" s="0" t="n">
-        <v>-109.791</v>
+        <v>-93.472</v>
       </c>
       <c r="D90" s="0" t="s">
         <v>53</v>
@@ -2015,16 +2139,16 @@
         <v>96</v>
       </c>
       <c r="B91" s="0" t="n">
-        <v>152.222</v>
+        <v>163.595</v>
       </c>
       <c r="C91" s="0" t="n">
-        <v>-109.791</v>
+        <v>-98.825</v>
       </c>
       <c r="D91" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E91" s="0" t="n">
-        <v>-90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2032,10 +2156,10 @@
         <v>97</v>
       </c>
       <c r="B92" s="0" t="n">
-        <v>147.32</v>
+        <v>125.0377</v>
       </c>
       <c r="C92" s="0" t="n">
-        <v>-109.791</v>
+        <v>-114.095</v>
       </c>
       <c r="D92" s="0" t="s">
         <v>53</v>
@@ -2049,10 +2173,10 @@
         <v>98</v>
       </c>
       <c r="B93" s="0" t="n">
-        <v>148.83</v>
+        <v>125.0377</v>
       </c>
       <c r="C93" s="0" t="n">
-        <v>-109.791</v>
+        <v>-121.545</v>
       </c>
       <c r="D93" s="0" t="s">
         <v>53</v>
@@ -2066,16 +2190,16 @@
         <v>99</v>
       </c>
       <c r="B94" s="0" t="n">
-        <v>139.225</v>
+        <v>173.5254</v>
       </c>
       <c r="C94" s="0" t="n">
-        <v>-117.71</v>
+        <v>-116.685</v>
       </c>
       <c r="D94" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E94" s="0" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2083,16 +2207,16 @@
         <v>100</v>
       </c>
       <c r="B95" s="0" t="n">
-        <v>139.225</v>
+        <v>173.5254</v>
       </c>
       <c r="C95" s="0" t="n">
-        <v>-116.2</v>
+        <v>-124.02</v>
       </c>
       <c r="D95" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E95" s="0" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2100,16 +2224,16 @@
         <v>101</v>
       </c>
       <c r="B96" s="0" t="n">
-        <v>143.6</v>
+        <v>153.137256</v>
       </c>
       <c r="C96" s="0" t="n">
-        <v>-112.575</v>
+        <v>-142.353171</v>
       </c>
       <c r="D96" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E96" s="0" t="n">
-        <v>-90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2117,16 +2241,16 @@
         <v>102</v>
       </c>
       <c r="B97" s="0" t="n">
-        <v>142.09</v>
+        <v>133.66</v>
       </c>
       <c r="C97" s="0" t="n">
-        <v>-112.575</v>
+        <v>-142.34</v>
       </c>
       <c r="D97" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E97" s="0" t="n">
-        <v>-90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2134,16 +2258,16 @@
         <v>103</v>
       </c>
       <c r="B98" s="0" t="n">
-        <v>159</v>
+        <v>143.54</v>
       </c>
       <c r="C98" s="0" t="n">
-        <v>-123.4</v>
+        <v>-142.34</v>
       </c>
       <c r="D98" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E98" s="0" t="n">
-        <v>90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2151,16 +2275,16 @@
         <v>104</v>
       </c>
       <c r="B99" s="0" t="n">
-        <v>158.75</v>
+        <v>122.3877</v>
       </c>
       <c r="C99" s="0" t="n">
-        <v>-117.729</v>
+        <v>-103.35</v>
       </c>
       <c r="D99" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E99" s="0" t="n">
-        <v>180</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2168,16 +2292,16 @@
         <v>105</v>
       </c>
       <c r="B100" s="0" t="n">
-        <v>157.4</v>
+        <v>122.3</v>
       </c>
       <c r="C100" s="0" t="n">
-        <v>-123.4</v>
+        <v>-129.9</v>
       </c>
       <c r="D100" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E100" s="0" t="n">
-        <v>90</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2185,10 +2309,10 @@
         <v>106</v>
       </c>
       <c r="B101" s="0" t="n">
-        <v>166.765</v>
+        <v>176.1675</v>
       </c>
       <c r="C101" s="0" t="n">
-        <v>-130.2</v>
+        <v>-108.25</v>
       </c>
       <c r="D101" s="0" t="s">
         <v>53</v>
@@ -2202,16 +2326,16 @@
         <v>107</v>
       </c>
       <c r="B102" s="0" t="n">
-        <v>169.8</v>
+        <v>176.1754</v>
       </c>
       <c r="C102" s="0" t="n">
-        <v>-120.625</v>
+        <v>-134.6</v>
       </c>
       <c r="D102" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E102" s="0" t="n">
-        <v>-90</v>
+        <v>90</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2219,16 +2343,16 @@
         <v>108</v>
       </c>
       <c r="B103" s="0" t="n">
-        <v>153.7</v>
+        <v>160.8</v>
       </c>
       <c r="C103" s="0" t="n">
-        <v>-102.525</v>
+        <v>-142.7</v>
       </c>
       <c r="D103" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E103" s="0" t="n">
-        <v>-90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2236,16 +2360,16 @@
         <v>109</v>
       </c>
       <c r="B104" s="0" t="n">
-        <v>167.25</v>
+        <v>134.116</v>
       </c>
       <c r="C104" s="0" t="n">
-        <v>-110.1</v>
+        <v>-98.716</v>
       </c>
       <c r="D104" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E104" s="0" t="n">
-        <v>-90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2253,16 +2377,16 @@
         <v>110</v>
       </c>
       <c r="B105" s="0" t="n">
-        <v>149.7226</v>
+        <v>157.103</v>
       </c>
       <c r="C105" s="0" t="n">
-        <v>-118.050315</v>
+        <v>-98.843</v>
       </c>
       <c r="D105" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E105" s="0" t="n">
-        <v>90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2270,10 +2394,10 @@
         <v>111</v>
       </c>
       <c r="B106" s="0" t="n">
-        <v>162.575</v>
+        <v>131.2</v>
       </c>
       <c r="C106" s="0" t="n">
-        <v>-102.975</v>
+        <v>-130.389</v>
       </c>
       <c r="D106" s="0" t="s">
         <v>53</v>
@@ -2287,16 +2411,16 @@
         <v>112</v>
       </c>
       <c r="B107" s="0" t="n">
-        <v>125.0377</v>
+        <v>131.182</v>
       </c>
       <c r="C107" s="0" t="n">
-        <v>-114.095</v>
+        <v>-112.732</v>
       </c>
       <c r="D107" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E107" s="0" t="n">
-        <v>-90</v>
+        <v>90</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2304,16 +2428,16 @@
         <v>113</v>
       </c>
       <c r="B108" s="0" t="n">
-        <v>125.0377</v>
+        <v>142.502711</v>
       </c>
       <c r="C108" s="0" t="n">
-        <v>-121.545</v>
+        <v>-125.867636</v>
       </c>
       <c r="D108" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E108" s="0" t="n">
-        <v>-90</v>
+        <v>145</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2321,16 +2445,16 @@
         <v>114</v>
       </c>
       <c r="B109" s="0" t="n">
-        <v>173.5254</v>
+        <v>142.748286</v>
       </c>
       <c r="C109" s="0" t="n">
-        <v>-124.02</v>
+        <v>-127.260364</v>
       </c>
       <c r="D109" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E109" s="0" t="n">
-        <v>90</v>
+        <v>145</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2338,16 +2462,16 @@
         <v>115</v>
       </c>
       <c r="B110" s="0" t="n">
-        <v>173.5254</v>
+        <v>140.69143</v>
       </c>
       <c r="C110" s="0" t="n">
-        <v>-116.685</v>
+        <v>-127.509966</v>
       </c>
       <c r="D110" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E110" s="0" t="n">
-        <v>90</v>
+        <v>-125</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2355,16 +2479,16 @@
         <v>116</v>
       </c>
       <c r="B111" s="0" t="n">
-        <v>141.893934</v>
+        <v>140.037166</v>
       </c>
       <c r="C111" s="0" t="n">
-        <v>-120.194788</v>
+        <v>-129.345506</v>
       </c>
       <c r="D111" s="0" t="s">
         <v>53</v>
       </c>
       <c r="E111" s="0" t="n">
-        <v>135</v>
+        <v>-125</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2372,15 +2496,712 @@
         <v>117</v>
       </c>
       <c r="B112" s="0" t="n">
-        <v>154.2</v>
+        <v>138.431152</v>
       </c>
       <c r="C112" s="0" t="n">
+        <v>-131.639132</v>
+      </c>
+      <c r="D112" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E112" s="0" t="n">
         <v>-125</v>
       </c>
-      <c r="D112" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="E112" s="0" t="n">
+    </row>
+    <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="B113" s="0" t="n">
+        <v>147</v>
+      </c>
+      <c r="C113" s="0" t="n">
+        <v>-128.4</v>
+      </c>
+      <c r="D113" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E113" s="0" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="B114" s="0" t="n">
+        <v>146.334967</v>
+      </c>
+      <c r="C114" s="0" t="n">
+        <v>-127.128441</v>
+      </c>
+      <c r="D114" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E114" s="0" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="B115" s="0" t="n">
+        <v>145.2</v>
+      </c>
+      <c r="C115" s="0" t="n">
+        <v>-129.4</v>
+      </c>
+      <c r="D115" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E115" s="0" t="n">
+        <v>-105</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="B116" s="0" t="n">
+        <v>144.8</v>
+      </c>
+      <c r="C116" s="0" t="n">
+        <v>-132.3</v>
+      </c>
+      <c r="D116" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E116" s="0" t="n">
+        <v>-105</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="B117" s="0" t="n">
+        <v>144.071425</v>
+      </c>
+      <c r="C117" s="0" t="n">
+        <v>-135.019081</v>
+      </c>
+      <c r="D117" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E117" s="0" t="n">
+        <v>-105</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="B118" s="0" t="n">
+        <v>147.469808</v>
+      </c>
+      <c r="C118" s="0" t="n">
+        <v>-124.84433</v>
+      </c>
+      <c r="D118" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E118" s="0" t="n">
+        <v>-105</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="B119" s="0" t="n">
+        <v>146.5</v>
+      </c>
+      <c r="C119" s="0" t="n">
+        <v>-124.6</v>
+      </c>
+      <c r="D119" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E119" s="0" t="n">
+        <v>-105</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="0" t="s">
+        <v>125</v>
+      </c>
+      <c r="B120" s="0" t="n">
+        <v>145</v>
+      </c>
+      <c r="C120" s="0" t="n">
+        <v>-135.3</v>
+      </c>
+      <c r="D120" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E120" s="0" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="B121" s="0" t="n">
+        <v>149.483691</v>
+      </c>
+      <c r="C121" s="0" t="n">
+        <v>-125.440827</v>
+      </c>
+      <c r="D121" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E121" s="0" t="n">
+        <v>-75</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="B122" s="0" t="n">
+        <v>150.449617</v>
+      </c>
+      <c r="C122" s="0" t="n">
+        <v>-125.182008</v>
+      </c>
+      <c r="D122" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E122" s="0" t="n">
+        <v>-75</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="B123" s="0" t="n">
+        <v>149.625776</v>
+      </c>
+      <c r="C123" s="0" t="n">
+        <v>-127.902947</v>
+      </c>
+      <c r="D123" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E123" s="0" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="B124" s="0" t="n">
+        <v>150.363502</v>
+      </c>
+      <c r="C124" s="0" t="n">
+        <v>-126.69588</v>
+      </c>
+      <c r="D124" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E124" s="0" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="0" t="s">
+        <v>130</v>
+      </c>
+      <c r="B125" s="0" t="n">
+        <v>151.437012</v>
+      </c>
+      <c r="C125" s="0" t="n">
+        <v>-128.867015</v>
+      </c>
+      <c r="D125" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E125" s="0" t="n">
+        <v>-75</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="B126" s="0" t="n">
+        <v>152.165587</v>
+      </c>
+      <c r="C126" s="0" t="n">
+        <v>-131.586096</v>
+      </c>
+      <c r="D126" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E126" s="0" t="n">
+        <v>-75</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="B127" s="0" t="n">
+        <v>152.45</v>
+      </c>
+      <c r="C127" s="0" t="n">
+        <v>-134.409491</v>
+      </c>
+      <c r="D127" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E127" s="0" t="n">
+        <v>-75</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="0" t="s">
+        <v>133</v>
+      </c>
+      <c r="B128" s="0" t="n">
+        <v>150.229854</v>
+      </c>
+      <c r="C128" s="0" t="n">
+        <v>-132.089245</v>
+      </c>
+      <c r="D128" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E128" s="0" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="B129" s="0" t="n">
+        <v>139.7</v>
+      </c>
+      <c r="C129" s="0" t="n">
+        <v>-112.649</v>
+      </c>
+      <c r="D129" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E129" s="0" t="n">
+        <v>-45</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="B130" s="0" t="n">
+        <v>138.557</v>
+      </c>
+      <c r="C130" s="0" t="n">
+        <v>-113.792</v>
+      </c>
+      <c r="D130" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E130" s="0" t="n">
+        <v>-45</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="0" t="s">
+        <v>136</v>
+      </c>
+      <c r="B131" s="0" t="n">
+        <v>158.6</v>
+      </c>
+      <c r="C131" s="0" t="n">
+        <v>-126.2</v>
+      </c>
+      <c r="D131" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E131" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="B132" s="0" t="n">
+        <v>150.622</v>
+      </c>
+      <c r="C132" s="0" t="n">
+        <v>-109.791</v>
+      </c>
+      <c r="D132" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E132" s="0" t="n">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="B133" s="0" t="n">
+        <v>152.222</v>
+      </c>
+      <c r="C133" s="0" t="n">
+        <v>-109.791</v>
+      </c>
+      <c r="D133" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E133" s="0" t="n">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="B134" s="0" t="n">
+        <v>147.32</v>
+      </c>
+      <c r="C134" s="0" t="n">
+        <v>-109.791</v>
+      </c>
+      <c r="D134" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E134" s="0" t="n">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="0" t="s">
+        <v>140</v>
+      </c>
+      <c r="B135" s="0" t="n">
+        <v>148.83</v>
+      </c>
+      <c r="C135" s="0" t="n">
+        <v>-109.791</v>
+      </c>
+      <c r="D135" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E135" s="0" t="n">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="B136" s="0" t="n">
+        <v>139.225</v>
+      </c>
+      <c r="C136" s="0" t="n">
+        <v>-117.71</v>
+      </c>
+      <c r="D136" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E136" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="0" t="s">
+        <v>142</v>
+      </c>
+      <c r="B137" s="0" t="n">
+        <v>139.225</v>
+      </c>
+      <c r="C137" s="0" t="n">
+        <v>-116.2</v>
+      </c>
+      <c r="D137" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E137" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="B138" s="0" t="n">
+        <v>143.6</v>
+      </c>
+      <c r="C138" s="0" t="n">
+        <v>-112.575</v>
+      </c>
+      <c r="D138" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E138" s="0" t="n">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="B139" s="0" t="n">
+        <v>142.09</v>
+      </c>
+      <c r="C139" s="0" t="n">
+        <v>-112.575</v>
+      </c>
+      <c r="D139" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E139" s="0" t="n">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="0" t="s">
+        <v>145</v>
+      </c>
+      <c r="B140" s="0" t="n">
+        <v>159</v>
+      </c>
+      <c r="C140" s="0" t="n">
+        <v>-123.4</v>
+      </c>
+      <c r="D140" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E140" s="0" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="B141" s="0" t="n">
+        <v>158.75</v>
+      </c>
+      <c r="C141" s="0" t="n">
+        <v>-117.729</v>
+      </c>
+      <c r="D141" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E141" s="0" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="B142" s="0" t="n">
+        <v>157.4</v>
+      </c>
+      <c r="C142" s="0" t="n">
+        <v>-123.4</v>
+      </c>
+      <c r="D142" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E142" s="0" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="B143" s="0" t="n">
+        <v>166.765</v>
+      </c>
+      <c r="C143" s="0" t="n">
+        <v>-130.2</v>
+      </c>
+      <c r="D143" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E143" s="0" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="B144" s="0" t="n">
+        <v>169.8</v>
+      </c>
+      <c r="C144" s="0" t="n">
+        <v>-120.625</v>
+      </c>
+      <c r="D144" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E144" s="0" t="n">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="B145" s="0" t="n">
+        <v>153.7</v>
+      </c>
+      <c r="C145" s="0" t="n">
+        <v>-102.525</v>
+      </c>
+      <c r="D145" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E145" s="0" t="n">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="B146" s="0" t="n">
+        <v>167.25</v>
+      </c>
+      <c r="C146" s="0" t="n">
+        <v>-110.1</v>
+      </c>
+      <c r="D146" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E146" s="0" t="n">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="B147" s="0" t="n">
+        <v>168.9</v>
+      </c>
+      <c r="C147" s="0" t="n">
+        <v>-117.7</v>
+      </c>
+      <c r="D147" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E147" s="0" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="B148" s="0" t="n">
+        <v>167</v>
+      </c>
+      <c r="C148" s="0" t="n">
+        <v>-107.1</v>
+      </c>
+      <c r="D148" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E148" s="0" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="B149" s="0" t="n">
+        <v>156.3</v>
+      </c>
+      <c r="C149" s="0" t="n">
+        <v>-103.1</v>
+      </c>
+      <c r="D149" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E149" s="0" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="0" t="s">
+        <v>155</v>
+      </c>
+      <c r="B150" s="0" t="n">
+        <v>149.7226</v>
+      </c>
+      <c r="C150" s="0" t="n">
+        <v>-118.050315</v>
+      </c>
+      <c r="D150" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E150" s="0" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="0" t="s">
+        <v>156</v>
+      </c>
+      <c r="B151" s="0" t="n">
+        <v>162.575</v>
+      </c>
+      <c r="C151" s="0" t="n">
+        <v>-102.975</v>
+      </c>
+      <c r="D151" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E151" s="0" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A152" s="0" t="s">
+        <v>157</v>
+      </c>
+      <c r="B152" s="0" t="n">
+        <v>141.893934</v>
+      </c>
+      <c r="C152" s="0" t="n">
+        <v>-120.194788</v>
+      </c>
+      <c r="D152" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E152" s="0" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="0" t="s">
+        <v>158</v>
+      </c>
+      <c r="B153" s="0" t="n">
+        <v>153.65</v>
+      </c>
+      <c r="C153" s="0" t="n">
+        <v>-124.45</v>
+      </c>
+      <c r="D153" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E153" s="0" t="n">
         <v>-145</v>
       </c>
     </row>

</xml_diff>